<commit_message>
Updated booking flow and API changes
</commit_message>
<xml_diff>
--- a/data/designs.xlsx
+++ b/data/designs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shyam\Desktop\EventDecor\event-decoration-site\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED2DB25-7E51-4921-9610-88378457E8BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368741E0-D245-4D83-82FE-B42F819F8F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="40">
   <si>
     <t>id</t>
   </si>
@@ -52,12 +52,6 @@
     <t>birthday</t>
   </si>
   <si>
-    <t>male</t>
-  </si>
-  <si>
-    <t>all</t>
-  </si>
-  <si>
     <t>Boss Baby Setup</t>
   </si>
   <si>
@@ -70,9 +64,6 @@
     <t>boss baby</t>
   </si>
   <si>
-    <t>https://objectstorage.ap-mumbai-1.oraclecloud.com/p/JaZ4VVLq8rPAZFGUnrXvYlPQQa3GPmYfU3ujEBRNK1Ab1AVjrOazTA2HTjURDEWj/n/bmd455xcti4w/b/Birthday/o/1_2ChicDecor1_2ChicDecor.png</t>
-  </si>
-  <si>
     <t>https://objectstorage.ap-mumbai-1.oraclecloud.com/p/o3U4nMAOUoqCBkDpdk6Gt-eNUDEGjPJKnaHedPWcAQE-lyUIVJxK7XN7t183wBqR/n/bmd455xcti4w/b/Birthday/o/1_1paw_patrol1_1paw_patrol.jpg</t>
   </si>
   <si>
@@ -143,6 +134,12 @@
   </si>
   <si>
     <t>https://objectstorage.ap-mumbai-1.oraclecloud.com/p/qDSlCXIrg1qdPEURLaLB9WXCWxapsyYHR_TAYy-RmYaP-CvwO4qMyVDzcJue6CBg/n/bmd455xcti4w/b/Birthday/o/InfantInfant_Bubble_Trouble_Balloon%20.jpg</t>
+  </si>
+  <si>
+    <t>https://objectstorage.ap-mumbai-1.oraclecloud.com/p/A8OflrQe9KbmKkAt4BTqkKDn83Z6BvCyt93SL2cMBy3SeWm_N3Xcay3Ts-cGfFN-/n/bmd455xcti4w/b/Birthday/o/Infantboss_baby.jpg</t>
+  </si>
+  <si>
+    <t>All</t>
   </si>
 </sst>
 </file>
@@ -416,7 +413,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>7</v>
@@ -430,26 +427,26 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D2" s="3">
-        <v>5499</v>
+        <v>2700</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>35</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>9</v>
@@ -460,28 +457,28 @@
         <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D3" s="3">
         <v>2500</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>9</v>
@@ -492,28 +489,28 @@
         <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D4" s="3">
         <v>2500</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>9</v>
@@ -524,25 +521,28 @@
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D5" s="3">
         <v>2500</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>9</v>
@@ -553,28 +553,28 @@
         <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D6" s="3">
         <v>2500</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="H6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>9</v>
@@ -585,28 +585,28 @@
         <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D7" s="3">
         <v>2600</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>9</v>
@@ -617,28 +617,28 @@
         <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D8" s="3">
         <v>1700</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F8" t="s">
-        <v>38</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="H8" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>9</v>

</xml_diff>